<commit_message>
feat: add reasoning benchmark queries
</commit_message>
<xml_diff>
--- a/docs-other-outputs/Gabay-RAG-140-Benchmark-Queries.xlsx
+++ b/docs-other-outputs/Gabay-RAG-140-Benchmark-Queries.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Retrieval'!$A$1:$H$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Response'!$A$1:$H$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reasoning'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reasoning'!$A$1:$H$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Report'!$A$1:$H$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4735,7 +4735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4780,8 +4780,848 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>REA-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>What is the course code and title of the published introductory programming course?</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Courses</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>RAG Courses</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>course</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Es et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>REA-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>List the published modules available in the introductory programming course.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>RAG Learning</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>module</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Es et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REA-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Who is the faculty member assigned to the Computer Science department and what are their contact details?</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>RAG People</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>user_directory</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Es et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>REA-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Show my current course grades for this term. My student ID is STU-2024-001.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Progress</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>RAG Progress</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>course_grade</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Es et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>REA-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Find the published database management course, then list its open sections with seat availability.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Courses</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>RAG Courses</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>course_section</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>REA-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Show my pending enrollment request, then trace its approval status and prerequisite requirements.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Courses</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>RAG Courses</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>enrollment_request</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>REA-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>List the published modules for the web development course, then show the items contained in each module.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>RAG Learning</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>module_item</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>REA-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Find the graded activities due before the midterm, then summarize their grading criteria from the published rubrics.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>RAG Learning</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>activity</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>REA-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Find the faculty members in the Information Technology department, then list their office hours and consultation schedules.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>RAG People</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>user_directory</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>REA-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>List the academic calendar events scheduled for October, then identify which ones are relevant to second-year students.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>RAG People</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>calendar_event</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>REA-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Retrieve my current grades across enrolled courses, then break them down by assessment component. My student ID is STU-2024-001.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Progress</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>RAG Progress</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>course_grade</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>REA-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>For each published programming course, identify its assigned instructor and their consultation schedule.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Courses</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>RAG Courses</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>course</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>REA-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>List my overdue learning activities across enrolled courses and show how each affects my current grades. My student ID is STU-2024-001.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>RAG Learning</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>activity</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>REA-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>For the published database management course, list its open sections and the published modules that cover its topics.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Courses</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>RAG Courses</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>course_section</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>REA-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Identify my instructors for this term and summarize the grades they have given me in their courses. My student ID is STU-2024-001.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>RAG People</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>user_directory</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>REA-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>List my enrolled courses with their section schedules, together with my current grade in each course. My student ID is STU-2024-001.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Courses</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>RAG Courses</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>course_section</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>REA-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Summarize the deadline-extension announcements across my enrolled courses and identify the instructor who posted each one.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>RAG Learning</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>announcement</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy + Multi-Step Pass Rate</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026; Chen et al. 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>REA-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>What is the capital city of Germany and what is its current population?</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Coordinator-direct</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>none (refusal)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>REA-19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Write a Python function that sorts a list of numbers using a custom sorting algorithm with full working code.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Coordinator-direct</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>none (refusal)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>REA-20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Who won the most recent Super Bowl championship and what was the final score?</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Coordinator-direct</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>none (refusal)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Agent Routing Accuracy</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Park &amp; Kwon 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:H21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add report queries complete 140 benchmark
</commit_message>
<xml_diff>
--- a/docs-other-outputs/Gabay-RAG-140-Benchmark-Queries.xlsx
+++ b/docs-other-outputs/Gabay-RAG-140-Benchmark-Queries.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Retrieval'!$A$1:$H$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Response'!$A$1:$H$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reasoning'!$A$1:$H$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Report'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Report'!$A$1:$H$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5632,7 +5632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5677,8 +5677,848 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>REP-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Generate a table of all published courses showing course code and title.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Courses</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Analytical Count</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>course</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>REP-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Generate a table of the published modules in the introductory programming course showing titles in order.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Analytical Count</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>module</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REP-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Generate a table of upcoming academic calendar events showing event name, date, and venue.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Analytical Count</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>calendar_event</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>REP-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Generate a table of my current grades across enrolled courses showing course code and grade. My student ID is STU-2024-001.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Progress</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Analytical Count</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>course_grade</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>REP-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Generate a table of open sections of the database management course showing schedule and available slots.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Courses</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Analytical Count</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>course_section</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>REP-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Generate a table of graded learning activities due before the midterm showing title, due date, and grading criteria.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>activity</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>REP-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Generate a summary table of my recorded quiz scores for the networking module showing attempt date and score without inferring missing attempts. My student ID is STU-2024-001.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>quiz</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>REP-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Generate a table of faculty members in the Information Technology department showing name, role, and office hours.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Analytical Count</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>user_directory</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>REP-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Generate a summary table of pending enrollment requests submitted in the last seven days showing request date and current status.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Courses</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>enrollment_request</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>REP-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Generate a summary table of course-related messages received grouped by sender role showing counts only without message content.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>message_meta</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>REP-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>For each published programming course, generate a comparison table of open sections showing schedule, seat availability, and instructor.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Courses</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>course_section</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Schema Adherence</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026; Baswardono et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>REP-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Generate a table of overdue learning activities across my enrolled courses showing due date, resubmission terms, and grade impact. My student ID is STU-2024-001.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>activity</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Schema Adherence</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026; Baswardono et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>REP-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Generate a table breaking down my current grades by assessment component across all enrolled courses. My student ID is STU-2024-001.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Progress</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>course_grade</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Schema Adherence</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026; Baswardono et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>REP-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>For each department offering courses this term, generate a table of assigned faculty members showing consultation schedules.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>user_directory</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Schema Adherence</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026; Baswardono et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>REP-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Generate a table mapping each of my final examinations to its review module showing coverage topics and exam dates.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>exam</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Schema Adherence</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026; Baswardono et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>REP-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Consolidate every deadline-extension announcement across my enrolled courses into one table showing course, new deadline, and effective date.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Learning</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>announcement</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Schema Adherence</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026; Baswardono et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>REP-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Generate a financial earnings report table for the top technology companies with quarterly revenue figures.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Coordinator-direct</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>none (refusal)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>REP-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Generate a league standings table for the professional basketball season with win-loss records and scores.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Coordinator-direct</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>none (refusal)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>REP-19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Generate a table deleting all enrollment request records and showing the removed entries.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Coordinator-direct</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>none (refusal)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>REP-20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Generate a gradebook table raising all student grades to passing marks before the deadline.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Coordinator-direct</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>none (refusal)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Data Consistency Rate</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Tiwari et al. 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:H21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>